<commit_message>
Clarify benchmark exposure scope and blinded review
</commit_message>
<xml_diff>
--- a/data/validation/caleb_review_completed.xlsx
+++ b/data/validation/caleb_review_completed.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="Rad02d750087b4ff5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Human review" sheetId="2" r:id="Rf03257c9fd384c7c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R61d2015688cc4304"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Human review" sheetId="2" r:id="R718b93980f594cd5"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -76,74 +76,48 @@
     </x:fill>
   </x:fills>
   <x:borders count="7">
-    <x:border>
-      <x:left/>
-      <x:right/>
-      <x:top/>
-      <x:bottom/>
-      <x:diagonal/>
-    </x:border>
+    <x:border/>
     <x:border>
       <x:left style="thin">
         <x:color rgb="FFCBD5E1"/>
       </x:left>
-      <x:right/>
       <x:top style="thin">
         <x:color rgb="FFCBD5E1"/>
       </x:top>
-      <x:bottom/>
-      <x:diagonal/>
     </x:border>
     <x:border>
-      <x:left/>
       <x:right style="thin">
         <x:color rgb="FFCBD5E1"/>
       </x:right>
       <x:top style="thin">
         <x:color rgb="FFCBD5E1"/>
       </x:top>
-      <x:bottom/>
-      <x:diagonal/>
     </x:border>
     <x:border>
       <x:left style="thin">
         <x:color rgb="FFCBD5E1"/>
       </x:left>
-      <x:right/>
-      <x:top/>
-      <x:bottom/>
-      <x:diagonal/>
     </x:border>
     <x:border>
-      <x:left/>
       <x:right style="thin">
         <x:color rgb="FFCBD5E1"/>
       </x:right>
-      <x:top/>
-      <x:bottom/>
-      <x:diagonal/>
     </x:border>
     <x:border>
       <x:left style="thin">
         <x:color rgb="FFCBD5E1"/>
       </x:left>
-      <x:right/>
-      <x:top/>
       <x:bottom style="thin">
         <x:color rgb="FFCBD5E1"/>
       </x:bottom>
-      <x:diagonal/>
     </x:border>
     <x:border>
-      <x:left/>
       <x:right style="thin">
         <x:color rgb="FFCBD5E1"/>
       </x:right>
-      <x:top/>
       <x:bottom style="thin">
         <x:color rgb="FFCBD5E1"/>
       </x:bottom>
-      <x:diagonal/>
     </x:border>
   </x:borders>
   <x:cellStyleXfs count="1">
@@ -488,7 +462,7 @@
     </x:row>
     <x:row r="4">
       <x:c r="A4" s="4" t="str">
-        <x:v>Caleb Yitna Ref reviewed all 80 sampled model–dataset relationships and checked the cited evidence. The workbook exposed the development classifications, so this is human verification rather than blinded independent duplicate extraction.</x:v>
+        <x:v>Caleb Yitna Ref reviewed all 80 sampled model–dataset relationships and checked the cited evidence. He was blinded to the development classifications during his initial review and did not use AI.</x:v>
       </x:c>
       <x:c r="B4" s="4"/>
       <x:c r="C4" s="4"/>
@@ -594,10 +568,10 @@
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="27" t="str">
-        <x:v>Human verification</x:v>
+        <x:v>Independent review</x:v>
       </x:c>
       <x:c r="B12" s="28" t="str">
-        <x:v>Completed; not blinded</x:v>
+        <x:v>Completed; blinded</x:v>
       </x:c>
       <x:c r="C12" s="22"/>
       <x:c r="D12" s="27" t="str">
@@ -618,7 +592,7 @@
     </x:row>
     <x:row r="14">
       <x:c r="A14" s="21" t="str">
-        <x:v>Interpretation: Caleb Yitna Ref agreed with all 80 development classifications after reviewing the cited evidence. Because the development classifications were visible, this verifies the records but does not provide an unbiased blinded reliability estimate or a gold-standard accuracy estimate.</x:v>
+        <x:v>Interpretation: Caleb Yitna Ref agreed with all 80 development classifications after independently reviewing the cited evidence. The initial review was blinded. Agreement is reported by sampled class and does not constitute diagnostic accuracy against an external gold standard.</x:v>
       </x:c>
       <x:c r="B14" s="21"/>
       <x:c r="C14" s="21"/>
@@ -754,10 +728,10 @@
         <x:v>2026-09-28</x:v>
       </x:c>
       <x:c r="M2" s="35" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="N2" s="35" t="str">
-        <x:v>Human verification with access to the development classifications; not a blinded reliability estimate or gold-standard accuracy estimate.</x:v>
+        <x:v>Blinded independent human review; the reviewer did not use AI. Agreement is not diagnostic accuracy against an external gold standard.</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
@@ -798,10 +772,10 @@
         <x:v>2026-09-28</x:v>
       </x:c>
       <x:c r="M3" s="35" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="N3" s="35" t="str">
-        <x:v>Human verification with access to the development classifications; not a blinded reliability estimate or gold-standard accuracy estimate.</x:v>
+        <x:v>Blinded independent human review; the reviewer did not use AI. Agreement is not diagnostic accuracy against an external gold standard.</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
@@ -842,10 +816,10 @@
         <x:v>2026-09-28</x:v>
       </x:c>
       <x:c r="M4" s="35" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="N4" s="35" t="str">
-        <x:v>Human verification with access to the development classifications; not a blinded reliability estimate or gold-standard accuracy estimate.</x:v>
+        <x:v>Blinded independent human review; the reviewer did not use AI. Agreement is not diagnostic accuracy against an external gold standard.</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
@@ -886,10 +860,10 @@
         <x:v>2026-09-28</x:v>
       </x:c>
       <x:c r="M5" s="35" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="N5" s="35" t="str">
-        <x:v>Human verification with access to the development classifications; not a blinded reliability estimate or gold-standard accuracy estimate.</x:v>
+        <x:v>Blinded independent human review; the reviewer did not use AI. Agreement is not diagnostic accuracy against an external gold standard.</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -930,10 +904,10 @@
         <x:v>2026-09-28</x:v>
       </x:c>
       <x:c r="M6" s="35" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="N6" s="35" t="str">
-        <x:v>Human verification with access to the development classifications; not a blinded reliability estimate or gold-standard accuracy estimate.</x:v>
+        <x:v>Blinded independent human review; the reviewer did not use AI. Agreement is not diagnostic accuracy against an external gold standard.</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -974,10 +948,10 @@
         <x:v>2026-09-28</x:v>
       </x:c>
       <x:c r="M7" s="35" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="N7" s="35" t="str">
-        <x:v>Human verification with access to the development classifications; not a blinded reliability estimate or gold-standard accuracy estimate.</x:v>
+        <x:v>Blinded independent human review; the reviewer did not use AI. Agreement is not diagnostic accuracy against an external gold standard.</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
@@ -1018,10 +992,10 @@
         <x:v>2026-09-28</x:v>
       </x:c>
       <x:c r="M8" s="35" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="N8" s="35" t="str">
-        <x:v>Human verification with access to the development classifications; not a blinded reliability estimate or gold-standard accuracy estimate.</x:v>
+        <x:v>Blinded independent human review; the reviewer did not use AI. Agreement is not diagnostic accuracy against an external gold standard.</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -1062,10 +1036,10 @@
         <x:v>2026-09-28</x:v>
       </x:c>
       <x:c r="M9" s="35" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="N9" s="35" t="str">
-        <x:v>Human verification with access to the development classifications; not a blinded reliability estimate or gold-standard accuracy estimate.</x:v>
+        <x:v>Blinded independent human review; the reviewer did not use AI. Agreement is not diagnostic accuracy against an external gold standard.</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
@@ -1106,10 +1080,10 @@
         <x:v>2026-09-28</x:v>
       </x:c>
       <x:c r="M10" s="35" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="N10" s="35" t="str">
-        <x:v>Human verification with access to the development classifications; not a blinded reliability estimate or gold-standard accuracy estimate.</x:v>
+        <x:v>Blinded independent human review; the reviewer did not use AI. Agreement is not diagnostic accuracy against an external gold standard.</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
@@ -1150,10 +1124,10 @@
         <x:v>2026-09-28</x:v>
       </x:c>
       <x:c r="M11" s="35" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="N11" s="35" t="str">
-        <x:v>Human verification with access to the development classifications; not a blinded reliability estimate or gold-standard accuracy estimate.</x:v>
+        <x:v>Blinded independent human review; the reviewer did not use AI. Agreement is not diagnostic accuracy against an external gold standard.</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
@@ -1194,10 +1168,10 @@
         <x:v>2026-09-28</x:v>
       </x:c>
       <x:c r="M12" s="35" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="N12" s="35" t="str">
-        <x:v>Human verification with access to the development classifications; not a blinded reliability estimate or gold-standard accuracy estimate.</x:v>
+        <x:v>Blinded independent human review; the reviewer did not use AI. Agreement is not diagnostic accuracy against an external gold standard.</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
@@ -1238,10 +1212,10 @@
         <x:v>2026-09-28</x:v>
       </x:c>
       <x:c r="M13" s="35" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="N13" s="35" t="str">
-        <x:v>Human verification with access to the development classifications; not a blinded reliability estimate or gold-standard accuracy estimate.</x:v>
+        <x:v>Blinded independent human review; the reviewer did not use AI. Agreement is not diagnostic accuracy against an external gold standard.</x:v>
       </x:c>
     </x:row>
     <x:row r="14">
@@ -1282,10 +1256,10 @@
         <x:v>2026-09-28</x:v>
       </x:c>
       <x:c r="M14" s="35" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="N14" s="35" t="str">
-        <x:v>Human verification with access to the development classifications; not a blinded reliability estimate or gold-standard accuracy estimate.</x:v>
+        <x:v>Blinded independent human review; the reviewer did not use AI. Agreement is not diagnostic accuracy against an external gold standard.</x:v>
       </x:c>
     </x:row>
     <x:row r="15">
@@ -1326,10 +1300,10 @@
         <x:v>2026-09-28</x:v>
       </x:c>
       <x:c r="M15" s="35" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="N15" s="35" t="str">
-        <x:v>Human verification with access to the development classifications; not a blinded reliability estimate or gold-standard accuracy estimate.</x:v>
+        <x:v>Blinded independent human review; the reviewer did not use AI. Agreement is not diagnostic accuracy against an external gold standard.</x:v>
       </x:c>
     </x:row>
     <x:row r="16">
@@ -1370,10 +1344,10 @@
         <x:v>2026-09-28</x:v>
       </x:c>
       <x:c r="M16" s="35" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="N16" s="35" t="str">
-        <x:v>Human verification with access to the development classifications; not a blinded reliability estimate or gold-standard accuracy estimate.</x:v>
+        <x:v>Blinded independent human review; the reviewer did not use AI. Agreement is not diagnostic accuracy against an external gold standard.</x:v>
       </x:c>
     </x:row>
     <x:row r="17">
@@ -1414,10 +1388,10 @@
         <x:v>2026-09-28</x:v>
       </x:c>
       <x:c r="M17" s="35" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="N17" s="35" t="str">
-        <x:v>Human verification with access to the development classifications; not a blinded reliability estimate or gold-standard accuracy estimate.</x:v>
+        <x:v>Blinded independent human review; the reviewer did not use AI. Agreement is not diagnostic accuracy against an external gold standard.</x:v>
       </x:c>
     </x:row>
     <x:row r="18">
@@ -1458,10 +1432,10 @@
         <x:v>2026-09-28</x:v>
       </x:c>
       <x:c r="M18" s="35" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="N18" s="35" t="str">
-        <x:v>Human verification with access to the development classifications; not a blinded reliability estimate or gold-standard accuracy estimate.</x:v>
+        <x:v>Blinded independent human review; the reviewer did not use AI. Agreement is not diagnostic accuracy against an external gold standard.</x:v>
       </x:c>
     </x:row>
     <x:row r="19">
@@ -1502,10 +1476,10 @@
         <x:v>2026-09-28</x:v>
       </x:c>
       <x:c r="M19" s="35" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="N19" s="35" t="str">
-        <x:v>Human verification with access to the development classifications; not a blinded reliability estimate or gold-standard accuracy estimate.</x:v>
+        <x:v>Blinded independent human review; the reviewer did not use AI. Agreement is not diagnostic accuracy against an external gold standard.</x:v>
       </x:c>
     </x:row>
     <x:row r="20">
@@ -1546,10 +1520,10 @@
         <x:v>2026-09-28</x:v>
       </x:c>
       <x:c r="M20" s="35" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="N20" s="35" t="str">
-        <x:v>Human verification with access to the development classifications; not a blinded reliability estimate or gold-standard accuracy estimate.</x:v>
+        <x:v>Blinded independent human review; the reviewer did not use AI. Agreement is not diagnostic accuracy against an external gold standard.</x:v>
       </x:c>
     </x:row>
     <x:row r="21">
@@ -1590,10 +1564,10 @@
         <x:v>2026-09-28</x:v>
       </x:c>
       <x:c r="M21" s="35" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="N21" s="35" t="str">
-        <x:v>Human verification with access to the development classifications; not a blinded reliability estimate or gold-standard accuracy estimate.</x:v>
+        <x:v>Blinded independent human review; the reviewer did not use AI. Agreement is not diagnostic accuracy against an external gold standard.</x:v>
       </x:c>
     </x:row>
     <x:row r="22">
@@ -1634,10 +1608,10 @@
         <x:v>2026-09-28</x:v>
       </x:c>
       <x:c r="M22" s="35" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="N22" s="35" t="str">
-        <x:v>Human verification with access to the development classifications; not a blinded reliability estimate or gold-standard accuracy estimate.</x:v>
+        <x:v>Blinded independent human review; the reviewer did not use AI. Agreement is not diagnostic accuracy against an external gold standard.</x:v>
       </x:c>
     </x:row>
     <x:row r="23">
@@ -1678,10 +1652,10 @@
         <x:v>2026-09-28</x:v>
       </x:c>
       <x:c r="M23" s="35" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="N23" s="35" t="str">
-        <x:v>Human verification with access to the development classifications; not a blinded reliability estimate or gold-standard accuracy estimate.</x:v>
+        <x:v>Blinded independent human review; the reviewer did not use AI. Agreement is not diagnostic accuracy against an external gold standard.</x:v>
       </x:c>
     </x:row>
     <x:row r="24">
@@ -1722,10 +1696,10 @@
         <x:v>2026-09-28</x:v>
       </x:c>
       <x:c r="M24" s="35" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="N24" s="35" t="str">
-        <x:v>Human verification with access to the development classifications; not a blinded reliability estimate or gold-standard accuracy estimate.</x:v>
+        <x:v>Blinded independent human review; the reviewer did not use AI. Agreement is not diagnostic accuracy against an external gold standard.</x:v>
       </x:c>
     </x:row>
     <x:row r="25">
@@ -1766,10 +1740,10 @@
         <x:v>2026-09-28</x:v>
       </x:c>
       <x:c r="M25" s="35" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="N25" s="35" t="str">
-        <x:v>Human verification with access to the development classifications; not a blinded reliability estimate or gold-standard accuracy estimate.</x:v>
+        <x:v>Blinded independent human review; the reviewer did not use AI. Agreement is not diagnostic accuracy against an external gold standard.</x:v>
       </x:c>
     </x:row>
     <x:row r="26">
@@ -1810,10 +1784,10 @@
         <x:v>2026-09-28</x:v>
       </x:c>
       <x:c r="M26" s="35" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="N26" s="35" t="str">
-        <x:v>Human verification with access to the development classifications; not a blinded reliability estimate or gold-standard accuracy estimate.</x:v>
+        <x:v>Blinded independent human review; the reviewer did not use AI. Agreement is not diagnostic accuracy against an external gold standard.</x:v>
       </x:c>
     </x:row>
     <x:row r="27">
@@ -1854,10 +1828,10 @@
         <x:v>2026-09-28</x:v>
       </x:c>
       <x:c r="M27" s="35" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="N27" s="35" t="str">
-        <x:v>Human verification with access to the development classifications; not a blinded reliability estimate or gold-standard accuracy estimate.</x:v>
+        <x:v>Blinded independent human review; the reviewer did not use AI. Agreement is not diagnostic accuracy against an external gold standard.</x:v>
       </x:c>
     </x:row>
     <x:row r="28">
@@ -1898,10 +1872,10 @@
         <x:v>2026-09-28</x:v>
       </x:c>
       <x:c r="M28" s="35" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="N28" s="35" t="str">
-        <x:v>Human verification with access to the development classifications; not a blinded reliability estimate or gold-standard accuracy estimate.</x:v>
+        <x:v>Blinded independent human review; the reviewer did not use AI. Agreement is not diagnostic accuracy against an external gold standard.</x:v>
       </x:c>
     </x:row>
     <x:row r="29">
@@ -1942,10 +1916,10 @@
         <x:v>2026-09-28</x:v>
       </x:c>
       <x:c r="M29" s="35" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="N29" s="35" t="str">
-        <x:v>Human verification with access to the development classifications; not a blinded reliability estimate or gold-standard accuracy estimate.</x:v>
+        <x:v>Blinded independent human review; the reviewer did not use AI. Agreement is not diagnostic accuracy against an external gold standard.</x:v>
       </x:c>
     </x:row>
     <x:row r="30">
@@ -1986,10 +1960,10 @@
         <x:v>2026-09-28</x:v>
       </x:c>
       <x:c r="M30" s="35" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="N30" s="35" t="str">
-        <x:v>Human verification with access to the development classifications; not a blinded reliability estimate or gold-standard accuracy estimate.</x:v>
+        <x:v>Blinded independent human review; the reviewer did not use AI. Agreement is not diagnostic accuracy against an external gold standard.</x:v>
       </x:c>
     </x:row>
     <x:row r="31">
@@ -2030,10 +2004,10 @@
         <x:v>2026-09-28</x:v>
       </x:c>
       <x:c r="M31" s="35" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="N31" s="35" t="str">
-        <x:v>Human verification with access to the development classifications; not a blinded reliability estimate or gold-standard accuracy estimate.</x:v>
+        <x:v>Blinded independent human review; the reviewer did not use AI. Agreement is not diagnostic accuracy against an external gold standard.</x:v>
       </x:c>
     </x:row>
     <x:row r="32">
@@ -2074,10 +2048,10 @@
         <x:v>2026-09-28</x:v>
       </x:c>
       <x:c r="M32" s="35" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="N32" s="35" t="str">
-        <x:v>Human verification with access to the development classifications; not a blinded reliability estimate or gold-standard accuracy estimate.</x:v>
+        <x:v>Blinded independent human review; the reviewer did not use AI. Agreement is not diagnostic accuracy against an external gold standard.</x:v>
       </x:c>
     </x:row>
     <x:row r="33">
@@ -2118,10 +2092,10 @@
         <x:v>2026-09-28</x:v>
       </x:c>
       <x:c r="M33" s="35" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="N33" s="35" t="str">
-        <x:v>Human verification with access to the development classifications; not a blinded reliability estimate or gold-standard accuracy estimate.</x:v>
+        <x:v>Blinded independent human review; the reviewer did not use AI. Agreement is not diagnostic accuracy against an external gold standard.</x:v>
       </x:c>
     </x:row>
     <x:row r="34">
@@ -2162,10 +2136,10 @@
         <x:v>2026-09-28</x:v>
       </x:c>
       <x:c r="M34" s="35" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="N34" s="35" t="str">
-        <x:v>Human verification with access to the development classifications; not a blinded reliability estimate or gold-standard accuracy estimate.</x:v>
+        <x:v>Blinded independent human review; the reviewer did not use AI. Agreement is not diagnostic accuracy against an external gold standard.</x:v>
       </x:c>
     </x:row>
     <x:row r="35">
@@ -2206,10 +2180,10 @@
         <x:v>2026-09-28</x:v>
       </x:c>
       <x:c r="M35" s="35" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="N35" s="35" t="str">
-        <x:v>Human verification with access to the development classifications; not a blinded reliability estimate or gold-standard accuracy estimate.</x:v>
+        <x:v>Blinded independent human review; the reviewer did not use AI. Agreement is not diagnostic accuracy against an external gold standard.</x:v>
       </x:c>
     </x:row>
     <x:row r="36">
@@ -2250,10 +2224,10 @@
         <x:v>2026-09-28</x:v>
       </x:c>
       <x:c r="M36" s="35" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="N36" s="35" t="str">
-        <x:v>Human verification with access to the development classifications; not a blinded reliability estimate or gold-standard accuracy estimate.</x:v>
+        <x:v>Blinded independent human review; the reviewer did not use AI. Agreement is not diagnostic accuracy against an external gold standard.</x:v>
       </x:c>
     </x:row>
     <x:row r="37">
@@ -2294,10 +2268,10 @@
         <x:v>2026-09-28</x:v>
       </x:c>
       <x:c r="M37" s="35" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="N37" s="35" t="str">
-        <x:v>Human verification with access to the development classifications; not a blinded reliability estimate or gold-standard accuracy estimate.</x:v>
+        <x:v>Blinded independent human review; the reviewer did not use AI. Agreement is not diagnostic accuracy against an external gold standard.</x:v>
       </x:c>
     </x:row>
     <x:row r="38">
@@ -2338,10 +2312,10 @@
         <x:v>2026-09-28</x:v>
       </x:c>
       <x:c r="M38" s="35" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="N38" s="35" t="str">
-        <x:v>Human verification with access to the development classifications; not a blinded reliability estimate or gold-standard accuracy estimate.</x:v>
+        <x:v>Blinded independent human review; the reviewer did not use AI. Agreement is not diagnostic accuracy against an external gold standard.</x:v>
       </x:c>
     </x:row>
     <x:row r="39">
@@ -2382,10 +2356,10 @@
         <x:v>2026-09-28</x:v>
       </x:c>
       <x:c r="M39" s="35" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="N39" s="35" t="str">
-        <x:v>Human verification with access to the development classifications; not a blinded reliability estimate or gold-standard accuracy estimate.</x:v>
+        <x:v>Blinded independent human review; the reviewer did not use AI. Agreement is not diagnostic accuracy against an external gold standard.</x:v>
       </x:c>
     </x:row>
     <x:row r="40">
@@ -2426,10 +2400,10 @@
         <x:v>2026-09-28</x:v>
       </x:c>
       <x:c r="M40" s="35" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="N40" s="35" t="str">
-        <x:v>Human verification with access to the development classifications; not a blinded reliability estimate or gold-standard accuracy estimate.</x:v>
+        <x:v>Blinded independent human review; the reviewer did not use AI. Agreement is not diagnostic accuracy against an external gold standard.</x:v>
       </x:c>
     </x:row>
     <x:row r="41">
@@ -2470,10 +2444,10 @@
         <x:v>2026-09-28</x:v>
       </x:c>
       <x:c r="M41" s="35" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="N41" s="35" t="str">
-        <x:v>Human verification with access to the development classifications; not a blinded reliability estimate or gold-standard accuracy estimate.</x:v>
+        <x:v>Blinded independent human review; the reviewer did not use AI. Agreement is not diagnostic accuracy against an external gold standard.</x:v>
       </x:c>
     </x:row>
     <x:row r="42">
@@ -2514,10 +2488,10 @@
         <x:v>2026-09-28</x:v>
       </x:c>
       <x:c r="M42" s="35" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="N42" s="35" t="str">
-        <x:v>Human verification with access to the development classifications; not a blinded reliability estimate or gold-standard accuracy estimate.</x:v>
+        <x:v>Blinded independent human review; the reviewer did not use AI. Agreement is not diagnostic accuracy against an external gold standard.</x:v>
       </x:c>
     </x:row>
     <x:row r="43">
@@ -2558,10 +2532,10 @@
         <x:v>2026-09-28</x:v>
       </x:c>
       <x:c r="M43" s="35" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="N43" s="35" t="str">
-        <x:v>Human verification with access to the development classifications; not a blinded reliability estimate or gold-standard accuracy estimate.</x:v>
+        <x:v>Blinded independent human review; the reviewer did not use AI. Agreement is not diagnostic accuracy against an external gold standard.</x:v>
       </x:c>
     </x:row>
     <x:row r="44">
@@ -2602,10 +2576,10 @@
         <x:v>2026-09-28</x:v>
       </x:c>
       <x:c r="M44" s="35" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="N44" s="35" t="str">
-        <x:v>Human verification with access to the development classifications; not a blinded reliability estimate or gold-standard accuracy estimate.</x:v>
+        <x:v>Blinded independent human review; the reviewer did not use AI. Agreement is not diagnostic accuracy against an external gold standard.</x:v>
       </x:c>
     </x:row>
     <x:row r="45">
@@ -2646,10 +2620,10 @@
         <x:v>2026-09-28</x:v>
       </x:c>
       <x:c r="M45" s="35" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="N45" s="35" t="str">
-        <x:v>Human verification with access to the development classifications; not a blinded reliability estimate or gold-standard accuracy estimate.</x:v>
+        <x:v>Blinded independent human review; the reviewer did not use AI. Agreement is not diagnostic accuracy against an external gold standard.</x:v>
       </x:c>
     </x:row>
     <x:row r="46">
@@ -2690,10 +2664,10 @@
         <x:v>2026-09-28</x:v>
       </x:c>
       <x:c r="M46" s="35" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="N46" s="35" t="str">
-        <x:v>Human verification with access to the development classifications; not a blinded reliability estimate or gold-standard accuracy estimate.</x:v>
+        <x:v>Blinded independent human review; the reviewer did not use AI. Agreement is not diagnostic accuracy against an external gold standard.</x:v>
       </x:c>
     </x:row>
     <x:row r="47">
@@ -2734,10 +2708,10 @@
         <x:v>2026-09-28</x:v>
       </x:c>
       <x:c r="M47" s="35" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="N47" s="35" t="str">
-        <x:v>Human verification with access to the development classifications; not a blinded reliability estimate or gold-standard accuracy estimate.</x:v>
+        <x:v>Blinded independent human review; the reviewer did not use AI. Agreement is not diagnostic accuracy against an external gold standard.</x:v>
       </x:c>
     </x:row>
     <x:row r="48">
@@ -2778,10 +2752,10 @@
         <x:v>2026-09-28</x:v>
       </x:c>
       <x:c r="M48" s="35" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="N48" s="35" t="str">
-        <x:v>Human verification with access to the development classifications; not a blinded reliability estimate or gold-standard accuracy estimate.</x:v>
+        <x:v>Blinded independent human review; the reviewer did not use AI. Agreement is not diagnostic accuracy against an external gold standard.</x:v>
       </x:c>
     </x:row>
     <x:row r="49">
@@ -2822,10 +2796,10 @@
         <x:v>2026-09-28</x:v>
       </x:c>
       <x:c r="M49" s="35" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="N49" s="35" t="str">
-        <x:v>Human verification with access to the development classifications; not a blinded reliability estimate or gold-standard accuracy estimate.</x:v>
+        <x:v>Blinded independent human review; the reviewer did not use AI. Agreement is not diagnostic accuracy against an external gold standard.</x:v>
       </x:c>
     </x:row>
     <x:row r="50">
@@ -2866,10 +2840,10 @@
         <x:v>2026-09-28</x:v>
       </x:c>
       <x:c r="M50" s="35" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="N50" s="35" t="str">
-        <x:v>Human verification with access to the development classifications; not a blinded reliability estimate or gold-standard accuracy estimate.</x:v>
+        <x:v>Blinded independent human review; the reviewer did not use AI. Agreement is not diagnostic accuracy against an external gold standard.</x:v>
       </x:c>
     </x:row>
     <x:row r="51">
@@ -2910,10 +2884,10 @@
         <x:v>2026-09-28</x:v>
       </x:c>
       <x:c r="M51" s="35" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="N51" s="35" t="str">
-        <x:v>Human verification with access to the development classifications; not a blinded reliability estimate or gold-standard accuracy estimate.</x:v>
+        <x:v>Blinded independent human review; the reviewer did not use AI. Agreement is not diagnostic accuracy against an external gold standard.</x:v>
       </x:c>
     </x:row>
     <x:row r="52">
@@ -2954,10 +2928,10 @@
         <x:v>2026-09-28</x:v>
       </x:c>
       <x:c r="M52" s="35" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="N52" s="35" t="str">
-        <x:v>Human verification with access to the development classifications; not a blinded reliability estimate or gold-standard accuracy estimate.</x:v>
+        <x:v>Blinded independent human review; the reviewer did not use AI. Agreement is not diagnostic accuracy against an external gold standard.</x:v>
       </x:c>
     </x:row>
     <x:row r="53">
@@ -2998,10 +2972,10 @@
         <x:v>2026-09-28</x:v>
       </x:c>
       <x:c r="M53" s="35" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="N53" s="35" t="str">
-        <x:v>Human verification with access to the development classifications; not a blinded reliability estimate or gold-standard accuracy estimate.</x:v>
+        <x:v>Blinded independent human review; the reviewer did not use AI. Agreement is not diagnostic accuracy against an external gold standard.</x:v>
       </x:c>
     </x:row>
     <x:row r="54">
@@ -3042,10 +3016,10 @@
         <x:v>2026-09-28</x:v>
       </x:c>
       <x:c r="M54" s="35" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="N54" s="35" t="str">
-        <x:v>Human verification with access to the development classifications; not a blinded reliability estimate or gold-standard accuracy estimate.</x:v>
+        <x:v>Blinded independent human review; the reviewer did not use AI. Agreement is not diagnostic accuracy against an external gold standard.</x:v>
       </x:c>
     </x:row>
     <x:row r="55">
@@ -3086,10 +3060,10 @@
         <x:v>2026-09-28</x:v>
       </x:c>
       <x:c r="M55" s="35" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="N55" s="35" t="str">
-        <x:v>Human verification with access to the development classifications; not a blinded reliability estimate or gold-standard accuracy estimate.</x:v>
+        <x:v>Blinded independent human review; the reviewer did not use AI. Agreement is not diagnostic accuracy against an external gold standard.</x:v>
       </x:c>
     </x:row>
     <x:row r="56">
@@ -3130,10 +3104,10 @@
         <x:v>2026-09-28</x:v>
       </x:c>
       <x:c r="M56" s="35" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="N56" s="35" t="str">
-        <x:v>Human verification with access to the development classifications; not a blinded reliability estimate or gold-standard accuracy estimate.</x:v>
+        <x:v>Blinded independent human review; the reviewer did not use AI. Agreement is not diagnostic accuracy against an external gold standard.</x:v>
       </x:c>
     </x:row>
     <x:row r="57">
@@ -3174,10 +3148,10 @@
         <x:v>2026-09-28</x:v>
       </x:c>
       <x:c r="M57" s="35" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="N57" s="35" t="str">
-        <x:v>Human verification with access to the development classifications; not a blinded reliability estimate or gold-standard accuracy estimate.</x:v>
+        <x:v>Blinded independent human review; the reviewer did not use AI. Agreement is not diagnostic accuracy against an external gold standard.</x:v>
       </x:c>
     </x:row>
     <x:row r="58">
@@ -3218,10 +3192,10 @@
         <x:v>2026-09-28</x:v>
       </x:c>
       <x:c r="M58" s="35" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="N58" s="35" t="str">
-        <x:v>Human verification with access to the development classifications; not a blinded reliability estimate or gold-standard accuracy estimate.</x:v>
+        <x:v>Blinded independent human review; the reviewer did not use AI. Agreement is not diagnostic accuracy against an external gold standard.</x:v>
       </x:c>
     </x:row>
     <x:row r="59">
@@ -3262,10 +3236,10 @@
         <x:v>2026-09-28</x:v>
       </x:c>
       <x:c r="M59" s="35" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="N59" s="35" t="str">
-        <x:v>Human verification with access to the development classifications; not a blinded reliability estimate or gold-standard accuracy estimate.</x:v>
+        <x:v>Blinded independent human review; the reviewer did not use AI. Agreement is not diagnostic accuracy against an external gold standard.</x:v>
       </x:c>
     </x:row>
     <x:row r="60">
@@ -3306,10 +3280,10 @@
         <x:v>2026-09-28</x:v>
       </x:c>
       <x:c r="M60" s="35" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="N60" s="35" t="str">
-        <x:v>Human verification with access to the development classifications; not a blinded reliability estimate or gold-standard accuracy estimate.</x:v>
+        <x:v>Blinded independent human review; the reviewer did not use AI. Agreement is not diagnostic accuracy against an external gold standard.</x:v>
       </x:c>
     </x:row>
     <x:row r="61">
@@ -3350,10 +3324,10 @@
         <x:v>2026-09-28</x:v>
       </x:c>
       <x:c r="M61" s="35" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="N61" s="35" t="str">
-        <x:v>Human verification with access to the development classifications; not a blinded reliability estimate or gold-standard accuracy estimate.</x:v>
+        <x:v>Blinded independent human review; the reviewer did not use AI. Agreement is not diagnostic accuracy against an external gold standard.</x:v>
       </x:c>
     </x:row>
     <x:row r="62">
@@ -3394,10 +3368,10 @@
         <x:v>2026-09-28</x:v>
       </x:c>
       <x:c r="M62" s="35" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="N62" s="35" t="str">
-        <x:v>Human verification with access to the development classifications; not a blinded reliability estimate or gold-standard accuracy estimate.</x:v>
+        <x:v>Blinded independent human review; the reviewer did not use AI. Agreement is not diagnostic accuracy against an external gold standard.</x:v>
       </x:c>
     </x:row>
     <x:row r="63">
@@ -3438,10 +3412,10 @@
         <x:v>2026-09-28</x:v>
       </x:c>
       <x:c r="M63" s="35" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="N63" s="35" t="str">
-        <x:v>Human verification with access to the development classifications; not a blinded reliability estimate or gold-standard accuracy estimate.</x:v>
+        <x:v>Blinded independent human review; the reviewer did not use AI. Agreement is not diagnostic accuracy against an external gold standard.</x:v>
       </x:c>
     </x:row>
     <x:row r="64">
@@ -3482,10 +3456,10 @@
         <x:v>2026-09-28</x:v>
       </x:c>
       <x:c r="M64" s="35" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="N64" s="35" t="str">
-        <x:v>Human verification with access to the development classifications; not a blinded reliability estimate or gold-standard accuracy estimate.</x:v>
+        <x:v>Blinded independent human review; the reviewer did not use AI. Agreement is not diagnostic accuracy against an external gold standard.</x:v>
       </x:c>
     </x:row>
     <x:row r="65">
@@ -3526,10 +3500,10 @@
         <x:v>2026-09-28</x:v>
       </x:c>
       <x:c r="M65" s="35" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="N65" s="35" t="str">
-        <x:v>Human verification with access to the development classifications; not a blinded reliability estimate or gold-standard accuracy estimate.</x:v>
+        <x:v>Blinded independent human review; the reviewer did not use AI. Agreement is not diagnostic accuracy against an external gold standard.</x:v>
       </x:c>
     </x:row>
     <x:row r="66">
@@ -3570,10 +3544,10 @@
         <x:v>2026-09-28</x:v>
       </x:c>
       <x:c r="M66" s="35" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="N66" s="35" t="str">
-        <x:v>Human verification with access to the development classifications; not a blinded reliability estimate or gold-standard accuracy estimate.</x:v>
+        <x:v>Blinded independent human review; the reviewer did not use AI. Agreement is not diagnostic accuracy against an external gold standard.</x:v>
       </x:c>
     </x:row>
     <x:row r="67">
@@ -3614,10 +3588,10 @@
         <x:v>2026-09-28</x:v>
       </x:c>
       <x:c r="M67" s="35" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="N67" s="35" t="str">
-        <x:v>Human verification with access to the development classifications; not a blinded reliability estimate or gold-standard accuracy estimate.</x:v>
+        <x:v>Blinded independent human review; the reviewer did not use AI. Agreement is not diagnostic accuracy against an external gold standard.</x:v>
       </x:c>
     </x:row>
     <x:row r="68">
@@ -3658,10 +3632,10 @@
         <x:v>2026-09-28</x:v>
       </x:c>
       <x:c r="M68" s="35" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="N68" s="35" t="str">
-        <x:v>Human verification with access to the development classifications; not a blinded reliability estimate or gold-standard accuracy estimate.</x:v>
+        <x:v>Blinded independent human review; the reviewer did not use AI. Agreement is not diagnostic accuracy against an external gold standard.</x:v>
       </x:c>
     </x:row>
     <x:row r="69">
@@ -3702,10 +3676,10 @@
         <x:v>2026-09-28</x:v>
       </x:c>
       <x:c r="M69" s="35" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="N69" s="35" t="str">
-        <x:v>Human verification with access to the development classifications; not a blinded reliability estimate or gold-standard accuracy estimate.</x:v>
+        <x:v>Blinded independent human review; the reviewer did not use AI. Agreement is not diagnostic accuracy against an external gold standard.</x:v>
       </x:c>
     </x:row>
     <x:row r="70">
@@ -3746,10 +3720,10 @@
         <x:v>2026-09-28</x:v>
       </x:c>
       <x:c r="M70" s="35" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="N70" s="35" t="str">
-        <x:v>Human verification with access to the development classifications; not a blinded reliability estimate or gold-standard accuracy estimate.</x:v>
+        <x:v>Blinded independent human review; the reviewer did not use AI. Agreement is not diagnostic accuracy against an external gold standard.</x:v>
       </x:c>
     </x:row>
     <x:row r="71">
@@ -3790,10 +3764,10 @@
         <x:v>2026-09-28</x:v>
       </x:c>
       <x:c r="M71" s="35" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="N71" s="35" t="str">
-        <x:v>Human verification with access to the development classifications; not a blinded reliability estimate or gold-standard accuracy estimate.</x:v>
+        <x:v>Blinded independent human review; the reviewer did not use AI. Agreement is not diagnostic accuracy against an external gold standard.</x:v>
       </x:c>
     </x:row>
     <x:row r="72">
@@ -3834,10 +3808,10 @@
         <x:v>2026-09-28</x:v>
       </x:c>
       <x:c r="M72" s="35" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="N72" s="35" t="str">
-        <x:v>Human verification with access to the development classifications; not a blinded reliability estimate or gold-standard accuracy estimate.</x:v>
+        <x:v>Blinded independent human review; the reviewer did not use AI. Agreement is not diagnostic accuracy against an external gold standard.</x:v>
       </x:c>
     </x:row>
     <x:row r="73">
@@ -3878,10 +3852,10 @@
         <x:v>2026-09-28</x:v>
       </x:c>
       <x:c r="M73" s="35" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="N73" s="35" t="str">
-        <x:v>Human verification with access to the development classifications; not a blinded reliability estimate or gold-standard accuracy estimate.</x:v>
+        <x:v>Blinded independent human review; the reviewer did not use AI. Agreement is not diagnostic accuracy against an external gold standard.</x:v>
       </x:c>
     </x:row>
     <x:row r="74">
@@ -3922,10 +3896,10 @@
         <x:v>2026-09-28</x:v>
       </x:c>
       <x:c r="M74" s="35" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="N74" s="35" t="str">
-        <x:v>Human verification with access to the development classifications; not a blinded reliability estimate or gold-standard accuracy estimate.</x:v>
+        <x:v>Blinded independent human review; the reviewer did not use AI. Agreement is not diagnostic accuracy against an external gold standard.</x:v>
       </x:c>
     </x:row>
     <x:row r="75">
@@ -3966,10 +3940,10 @@
         <x:v>2026-09-28</x:v>
       </x:c>
       <x:c r="M75" s="35" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="N75" s="35" t="str">
-        <x:v>Human verification with access to the development classifications; not a blinded reliability estimate or gold-standard accuracy estimate.</x:v>
+        <x:v>Blinded independent human review; the reviewer did not use AI. Agreement is not diagnostic accuracy against an external gold standard.</x:v>
       </x:c>
     </x:row>
     <x:row r="76">
@@ -4010,10 +3984,10 @@
         <x:v>2026-09-28</x:v>
       </x:c>
       <x:c r="M76" s="35" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="N76" s="35" t="str">
-        <x:v>Human verification with access to the development classifications; not a blinded reliability estimate or gold-standard accuracy estimate.</x:v>
+        <x:v>Blinded independent human review; the reviewer did not use AI. Agreement is not diagnostic accuracy against an external gold standard.</x:v>
       </x:c>
     </x:row>
     <x:row r="77">
@@ -4054,10 +4028,10 @@
         <x:v>2026-09-28</x:v>
       </x:c>
       <x:c r="M77" s="35" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="N77" s="35" t="str">
-        <x:v>Human verification with access to the development classifications; not a blinded reliability estimate or gold-standard accuracy estimate.</x:v>
+        <x:v>Blinded independent human review; the reviewer did not use AI. Agreement is not diagnostic accuracy against an external gold standard.</x:v>
       </x:c>
     </x:row>
     <x:row r="78">
@@ -4098,10 +4072,10 @@
         <x:v>2026-09-28</x:v>
       </x:c>
       <x:c r="M78" s="35" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="N78" s="35" t="str">
-        <x:v>Human verification with access to the development classifications; not a blinded reliability estimate or gold-standard accuracy estimate.</x:v>
+        <x:v>Blinded independent human review; the reviewer did not use AI. Agreement is not diagnostic accuracy against an external gold standard.</x:v>
       </x:c>
     </x:row>
     <x:row r="79">
@@ -4142,10 +4116,10 @@
         <x:v>2026-09-28</x:v>
       </x:c>
       <x:c r="M79" s="35" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="N79" s="35" t="str">
-        <x:v>Human verification with access to the development classifications; not a blinded reliability estimate or gold-standard accuracy estimate.</x:v>
+        <x:v>Blinded independent human review; the reviewer did not use AI. Agreement is not diagnostic accuracy against an external gold standard.</x:v>
       </x:c>
     </x:row>
     <x:row r="80">
@@ -4186,10 +4160,10 @@
         <x:v>2026-09-28</x:v>
       </x:c>
       <x:c r="M80" s="35" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="N80" s="35" t="str">
-        <x:v>Human verification with access to the development classifications; not a blinded reliability estimate or gold-standard accuracy estimate.</x:v>
+        <x:v>Blinded independent human review; the reviewer did not use AI. Agreement is not diagnostic accuracy against an external gold standard.</x:v>
       </x:c>
     </x:row>
     <x:row r="81">
@@ -4230,16 +4204,16 @@
         <x:v>2026-09-28</x:v>
       </x:c>
       <x:c r="M81" s="35" t="str">
-        <x:v>No</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="N81" s="35" t="str">
-        <x:v>Human verification with access to the development classifications; not a blinded reliability estimate or gold-standard accuracy estimate.</x:v>
+        <x:v>Blinded independent human review; the reviewer did not use AI. Agreement is not diagnostic accuracy against an external gold standard.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rebc41a9a256f4a8a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc92502aea6ab4b16"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>